<commit_message>
all the same but without using anonymisering
</commit_message>
<xml_diff>
--- a/analysis/CBM/2025/Konte/data/results/IN1020_2025_CBM_konte_results.xlsx
+++ b/analysis/CBM/2025/Konte/data/results/IN1020_2025_CBM_konte_results.xlsx
@@ -517,13 +517,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>15262</v>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>-2</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
@@ -532,72 +532,72 @@
         <v>8</v>
       </c>
       <c r="F2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>8</v>
       </c>
       <c r="H2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K2" t="n">
+        <v>8</v>
+      </c>
+      <c r="L2" t="n">
+        <v>8</v>
+      </c>
+      <c r="M2" t="n">
         <v>0</v>
       </c>
-      <c r="J2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K2" t="n">
-        <v>8</v>
-      </c>
-      <c r="L2" t="n">
-        <v>8</v>
-      </c>
-      <c r="M2" t="n">
-        <v>4</v>
-      </c>
       <c r="N2" t="n">
         <v>4</v>
       </c>
       <c r="O2" t="n">
-        <v>6</v>
+        <v>-12</v>
       </c>
       <c r="P2" t="n">
         <v>8</v>
       </c>
       <c r="Q2" t="n">
-        <v>95</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>15263</v>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
         <v>8</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="G3" t="n">
         <v>8</v>
       </c>
       <c r="H3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J3" t="n">
-        <v>4</v>
+        <v>-6</v>
       </c>
       <c r="K3" t="n">
         <v>8</v>
@@ -606,41 +606,39 @@
         <v>8</v>
       </c>
       <c r="M3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N3" t="n">
-        <v>8</v>
+        <v>-6</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P3" t="n">
         <v>8</v>
       </c>
       <c r="Q3" t="n">
-        <v>84</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>15264</v>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
         <v>8</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+      <c r="F4" t="n">
+        <v>8</v>
       </c>
       <c r="G4" t="n">
         <v>8</v>
@@ -648,108 +646,96 @@
       <c r="H4" t="n">
         <v>8</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L4" t="n">
+        <v>7</v>
       </c>
       <c r="M4" t="n">
-        <v>8</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>7</v>
+      </c>
+      <c r="N4" t="n">
+        <v>8</v>
       </c>
       <c r="O4" t="n">
         <v>8</v>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+      <c r="P4" t="n">
+        <v>4</v>
       </c>
       <c r="Q4" t="n">
-        <v>56</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>15265</v>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>-7</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L5" t="n">
-        <v>8</v>
+        <v>-1</v>
       </c>
       <c r="M5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O5" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="P5" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q5" t="n">
-        <v>115</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>15266</v>
       </c>
       <c r="B6" t="n">
         <v>8</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
         <v>8</v>
@@ -758,19 +744,19 @@
         <v>8</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
         <v>8</v>
       </c>
       <c r="H6" t="n">
-        <v>-12</v>
+        <v>5</v>
       </c>
       <c r="I6" t="n">
         <v>8</v>
       </c>
       <c r="J6" t="n">
-        <v>8</v>
+        <v>-2</v>
       </c>
       <c r="K6" t="n">
         <v>8</v>
@@ -778,33 +764,31 @@
       <c r="L6" t="n">
         <v>8</v>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+      <c r="M6" t="n">
+        <v>5</v>
       </c>
       <c r="N6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="O6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="P6" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>15268</v>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C7" t="n">
-        <v>-2</v>
+        <v>8</v>
       </c>
       <c r="D7" t="n">
         <v>8</v>
@@ -819,54 +803,54 @@
         <v>8</v>
       </c>
       <c r="H7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L7" t="n">
         <v>8</v>
       </c>
       <c r="M7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P7" t="n">
         <v>8</v>
       </c>
       <c r="Q7" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>15270</v>
       </c>
       <c r="B8" t="n">
         <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E8" t="n">
         <v>8</v>
       </c>
       <c r="F8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G8" t="n">
         <v>8</v>
@@ -875,42 +859,42 @@
         <v>6</v>
       </c>
       <c r="I8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J8" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" t="n">
+        <v>8</v>
+      </c>
+      <c r="L8" t="n">
+        <v>6</v>
+      </c>
+      <c r="M8" t="n">
         <v>0</v>
       </c>
-      <c r="K8" t="n">
-        <v>8</v>
-      </c>
-      <c r="L8" t="n">
-        <v>8</v>
-      </c>
-      <c r="M8" t="n">
-        <v>6</v>
-      </c>
       <c r="N8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>103</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>15272</v>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
         <v>-12</v>
@@ -919,19 +903,19 @@
         <v>8</v>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="G9" t="n">
         <v>8</v>
       </c>
       <c r="H9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K9" t="n">
         <v>8</v>
@@ -940,24 +924,24 @@
         <v>8</v>
       </c>
       <c r="M9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O9" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="P9" t="n">
         <v>8</v>
       </c>
       <c r="Q9" t="n">
-        <v>91</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>15273</v>
       </c>
       <c r="B10" t="n">
         <v>8</v>
@@ -965,135 +949,129 @@
       <c r="C10" t="n">
         <v>8</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+      <c r="D10" t="n">
+        <v>4</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
       </c>
       <c r="F10" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
+        <v>8</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I10" t="n">
+        <v>8</v>
+      </c>
+      <c r="J10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" t="n">
+        <v>8</v>
+      </c>
+      <c r="M10" t="n">
         <v>0</v>
       </c>
-      <c r="H10" t="n">
-        <v>4</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>-12</v>
-      </c>
-      <c r="K10" t="n">
-        <v>-12</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
-        <v>4</v>
-      </c>
       <c r="N10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O10" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Q10" t="n">
-        <v>39</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>15274</v>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>-6</v>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
         <v>8</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G11" t="n">
         <v>8</v>
       </c>
       <c r="H11" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I11" t="n">
         <v>8</v>
       </c>
       <c r="J11" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K11" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="L11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M11" t="n">
-        <v>4</v>
+        <v>-7</v>
       </c>
       <c r="N11" t="n">
         <v>8</v>
       </c>
       <c r="O11" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="P11" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q11" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>15275</v>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
         <v>8</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>-12</v>
       </c>
       <c r="E12" t="n">
         <v>8</v>
       </c>
       <c r="F12" t="n">
-        <v>4</v>
+        <v>-12</v>
       </c>
       <c r="G12" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="H12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J12" t="n">
         <v>8</v>
@@ -1105,33 +1083,33 @@
         <v>8</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="N12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="O12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="P12" t="n">
         <v>4</v>
       </c>
       <c r="Q12" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>15276</v>
       </c>
       <c r="B13" t="n">
         <v>8</v>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E13" t="n">
         <v>8</v>
@@ -1143,149 +1121,149 @@
         <v>8</v>
       </c>
       <c r="H13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J13" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K13" t="n">
         <v>8</v>
       </c>
       <c r="L13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M13" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N13" t="n">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O13" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q13" t="n">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>15278</v>
       </c>
       <c r="B14" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D14" t="n">
-        <v>8</v>
+        <v>0</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="E14" t="n">
         <v>8</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G14" t="n">
         <v>8</v>
       </c>
       <c r="H14" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I14" t="n">
-        <v>7</v>
-      </c>
-      <c r="J14" t="n">
-        <v>8</v>
+        <v>8</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="K14" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L14" t="n">
-        <v>8</v>
+        <v>-1</v>
       </c>
       <c r="M14" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N14" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O14" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P14" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q14" t="n">
-        <v>111</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>15282</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>8</v>
+      </c>
+      <c r="D15" t="n">
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G15" t="n">
         <v>8</v>
       </c>
       <c r="H15" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I15" t="n">
         <v>8</v>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+      <c r="J15" t="n">
+        <v>8</v>
       </c>
       <c r="K15" t="n">
-        <v>3</v>
+        <v>-12</v>
       </c>
       <c r="L15" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O15" t="n">
-        <v>6</v>
+        <v>-12</v>
       </c>
       <c r="P15" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q15" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>15283</v>
       </c>
       <c r="B16" t="n">
         <v>7</v>
@@ -1294,19 +1272,19 @@
         <v>8</v>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
         <v>8</v>
       </c>
       <c r="F16" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G16" t="n">
         <v>8</v>
       </c>
       <c r="H16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I16" t="n">
         <v>8</v>
@@ -1315,7 +1293,7 @@
         <v>4</v>
       </c>
       <c r="K16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L16" t="n">
         <v>8</v>
@@ -1327,35 +1305,33 @@
         <v>8</v>
       </c>
       <c r="O16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P16" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>15284</v>
+      </c>
+      <c r="B17" t="n">
+        <v>8</v>
       </c>
       <c r="C17" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
         <v>8</v>
       </c>
       <c r="F17" t="n">
-        <v>8</v>
+        <v>-2</v>
       </c>
       <c r="G17" t="n">
         <v>8</v>
@@ -1364,95 +1340,101 @@
         <v>8</v>
       </c>
       <c r="I17" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J17" t="n">
-        <v>-12</v>
+        <v>6</v>
       </c>
       <c r="K17" t="n">
         <v>8</v>
       </c>
       <c r="L17" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="M17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N17" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O17" t="n">
-        <v>8</v>
+        <v>-3</v>
       </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q17" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>15286</v>
       </c>
       <c r="B18" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C18" t="n">
         <v>8</v>
       </c>
-      <c r="D18" t="n">
-        <v>8</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="E18" t="n">
         <v>8</v>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G18" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="H18" t="n">
-        <v>7</v>
-      </c>
-      <c r="I18" t="n">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="J18" t="n">
-        <v>-2</v>
+        <v>-12</v>
       </c>
       <c r="K18" t="n">
-        <v>7</v>
-      </c>
-      <c r="L18" t="n">
-        <v>8</v>
+        <v>-12</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="M18" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O18" t="n">
         <v>8</v>
       </c>
       <c r="P18" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q18" t="n">
-        <v>96</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>18</v>
+        <v>15288</v>
       </c>
       <c r="B19" t="n">
         <v>8</v>
       </c>
       <c r="C19" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
         <v>8</v>
@@ -1461,7 +1443,7 @@
         <v>8</v>
       </c>
       <c r="F19" t="n">
-        <v>8</v>
+        <v>-6</v>
       </c>
       <c r="G19" t="n">
         <v>8</v>
@@ -1482,30 +1464,32 @@
         <v>8</v>
       </c>
       <c r="M19" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="N19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O19" t="n">
         <v>8</v>
       </c>
       <c r="P19" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q19" t="n">
-        <v>116</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" t="n">
-        <v>4</v>
+        <v>15289</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="C20" t="n">
-        <v>-2</v>
+        <v>8</v>
       </c>
       <c r="D20" t="n">
         <v>8</v>
@@ -1514,19 +1498,19 @@
         <v>8</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G20" t="n">
         <v>8</v>
       </c>
       <c r="H20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I20" t="n">
         <v>4</v>
       </c>
       <c r="J20" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="K20" t="n">
         <v>8</v>
@@ -1535,48 +1519,48 @@
         <v>8</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N20" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="O20" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="P20" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="Q20" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>20</v>
+        <v>15290</v>
       </c>
       <c r="B21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
         <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E21" t="n">
         <v>8</v>
       </c>
       <c r="F21" t="n">
-        <v>-6</v>
+        <v>4</v>
       </c>
       <c r="G21" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="H21" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I21" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J21" t="n">
         <v>8</v>
@@ -1585,42 +1569,42 @@
         <v>8</v>
       </c>
       <c r="L21" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N21" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O21" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="P21" t="n">
         <v>8</v>
       </c>
       <c r="Q21" t="n">
-        <v>93</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>21</v>
+        <v>15291</v>
       </c>
       <c r="B22" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>6</v>
+        <v>-2</v>
       </c>
       <c r="D22" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E22" t="n">
         <v>8</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G22" t="n">
         <v>8</v>
@@ -1629,60 +1613,60 @@
         <v>8</v>
       </c>
       <c r="I22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K22" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L22" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="M22" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O22" t="n">
-        <v>-3</v>
+        <v>8</v>
       </c>
       <c r="P22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q22" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>22</v>
+        <v>15292</v>
       </c>
       <c r="B23" t="n">
         <v>8</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="E23" t="n">
         <v>8</v>
       </c>
       <c r="F23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G23" t="n">
         <v>8</v>
       </c>
       <c r="H23" t="n">
-        <v>6</v>
+        <v>-12</v>
       </c>
       <c r="I23" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J23" t="n">
         <v>8</v>
@@ -1693,87 +1677,89 @@
       <c r="L23" t="n">
         <v>8</v>
       </c>
-      <c r="M23" t="n">
-        <v>2</v>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="N23" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O23" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P23" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q23" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>23</v>
+        <v>15293</v>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C24" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D24" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G24" t="n">
         <v>8</v>
       </c>
       <c r="H24" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I24" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J24" t="n">
+        <v>5</v>
+      </c>
+      <c r="K24" t="n">
+        <v>8</v>
+      </c>
+      <c r="L24" t="n">
+        <v>8</v>
+      </c>
+      <c r="M24" t="n">
+        <v>8</v>
+      </c>
+      <c r="N24" t="n">
+        <v>6</v>
+      </c>
+      <c r="O24" t="n">
+        <v>7</v>
+      </c>
+      <c r="P24" t="n">
         <v>-2</v>
       </c>
-      <c r="K24" t="n">
-        <v>4</v>
-      </c>
-      <c r="L24" t="n">
-        <v>8</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>8</v>
-      </c>
-      <c r="O24" t="n">
-        <v>8</v>
-      </c>
-      <c r="P24" t="n">
-        <v>8</v>
-      </c>
       <c r="Q24" t="n">
-        <v>59</v>
+        <v>86</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>24</v>
+        <v>15294</v>
       </c>
       <c r="B25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D25" t="n">
-        <v>-6</v>
+        <v>-12</v>
       </c>
       <c r="E25" t="n">
         <v>8</v>
@@ -1785,160 +1771,160 @@
         <v>8</v>
       </c>
       <c r="H25" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J25" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="K25" t="n">
         <v>8</v>
       </c>
       <c r="L25" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="M25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N25" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="O25" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="P25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q25" t="n">
-        <v>93</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>25</v>
+        <v>15296</v>
       </c>
       <c r="B26" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
         <v>8</v>
       </c>
       <c r="D26" t="n">
-        <v>-12</v>
+        <v>4</v>
       </c>
       <c r="E26" t="n">
         <v>8</v>
       </c>
       <c r="F26" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="G26" t="n">
         <v>8</v>
       </c>
       <c r="H26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I26" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J26" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L26" t="n">
         <v>8</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O26" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P26" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q26" t="n">
-        <v>68</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>26</v>
+        <v>15297</v>
       </c>
       <c r="B27" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D27" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="E27" t="n">
         <v>8</v>
       </c>
       <c r="F27" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G27" t="n">
         <v>8</v>
       </c>
       <c r="H27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I27" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J27" t="n">
         <v>4</v>
       </c>
       <c r="K27" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L27" t="n">
         <v>8</v>
       </c>
       <c r="M27" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
         <v>8</v>
       </c>
       <c r="O27" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="P27" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q27" t="n">
-        <v>60</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>27</v>
+        <v>15298</v>
       </c>
       <c r="B28" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E28" t="n">
         <v>8</v>
       </c>
       <c r="F28" t="n">
-        <v>-3</v>
+        <v>5</v>
       </c>
       <c r="G28" t="n">
         <v>8</v>
@@ -1947,42 +1933,42 @@
         <v>4</v>
       </c>
       <c r="I28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J28" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K28" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L28" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M28" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="N28" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O28" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q28" t="n">
-        <v>71</v>
+        <v>97</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>28</v>
+        <v>15299</v>
       </c>
       <c r="B29" t="n">
-        <v>-2</v>
+        <v>5</v>
       </c>
       <c r="C29" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
         <v>-12</v>
@@ -1991,7 +1977,7 @@
         <v>8</v>
       </c>
       <c r="F29" t="n">
-        <v>7</v>
+        <v>-7</v>
       </c>
       <c r="G29" t="n">
         <v>8</v>
@@ -2000,21 +1986,19 @@
         <v>5</v>
       </c>
       <c r="I29" t="n">
-        <v>6</v>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>7</v>
+      </c>
+      <c r="J29" t="n">
+        <v>8</v>
       </c>
       <c r="K29" t="n">
         <v>8</v>
       </c>
       <c r="L29" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M29" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N29" t="n">
         <v>4</v>
@@ -2023,68 +2007,68 @@
         <v>6</v>
       </c>
       <c r="P29" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q29" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>29</v>
+        <v>15300</v>
       </c>
       <c r="B30" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C30" t="n">
-        <v>-12</v>
+        <v>4</v>
       </c>
       <c r="D30" t="n">
-        <v>-12</v>
+        <v>6</v>
       </c>
       <c r="E30" t="n">
         <v>8</v>
       </c>
       <c r="F30" t="n">
-        <v>-12</v>
+        <v>6</v>
       </c>
       <c r="G30" t="n">
         <v>8</v>
       </c>
       <c r="H30" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I30" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="J30" t="n">
         <v>8</v>
       </c>
       <c r="K30" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L30" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N30" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O30" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P30" t="n">
         <v>6</v>
       </c>
       <c r="Q30" t="n">
-        <v>47</v>
+        <v>82</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>30</v>
+        <v>15301</v>
       </c>
       <c r="B31" t="n">
         <v>8</v>
@@ -2093,7 +2077,7 @@
         <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E31" t="n">
         <v>8</v>
@@ -2105,54 +2089,54 @@
         <v>8</v>
       </c>
       <c r="H31" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I31" t="n">
         <v>6</v>
       </c>
       <c r="J31" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K31" t="n">
         <v>8</v>
       </c>
       <c r="L31" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M31" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N31" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P31" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q31" t="n">
-        <v>89</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>31</v>
+        <v>15302</v>
       </c>
       <c r="B32" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C32" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D32" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="E32" t="n">
         <v>8</v>
       </c>
       <c r="F32" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G32" t="n">
         <v>8</v>
@@ -2164,148 +2148,174 @@
         <v>8</v>
       </c>
       <c r="J32" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K32" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L32" t="n">
         <v>8</v>
       </c>
       <c r="M32" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O32" t="n">
         <v>8</v>
       </c>
       <c r="P32" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="Q32" t="n">
-        <v>97</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>32</v>
+        <v>15303</v>
       </c>
       <c r="B33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C33" t="n">
         <v>6</v>
       </c>
       <c r="D33" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H33" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I33" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J33" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K33" t="n">
         <v>8</v>
       </c>
       <c r="L33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N33" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="P33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q33" t="n">
-        <v>71</v>
+        <v>115</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" t="n">
-        <v>7</v>
-      </c>
-      <c r="C34" t="n">
-        <v>-7</v>
-      </c>
-      <c r="D34" t="n">
-        <v>5</v>
+        <v>15304</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="E34" t="n">
-        <v>5</v>
-      </c>
-      <c r="F34" t="n">
-        <v>6</v>
-      </c>
-      <c r="G34" t="n">
-        <v>3</v>
-      </c>
-      <c r="H34" t="n">
-        <v>5</v>
-      </c>
-      <c r="I34" t="n">
-        <v>7</v>
-      </c>
-      <c r="J34" t="n">
-        <v>6</v>
-      </c>
-      <c r="K34" t="n">
-        <v>4</v>
-      </c>
-      <c r="L34" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="M34" t="n">
-        <v>5</v>
-      </c>
-      <c r="N34" t="n">
-        <v>7</v>
-      </c>
-      <c r="O34" t="n">
-        <v>5</v>
-      </c>
-      <c r="P34" t="n">
-        <v>5</v>
+        <v>-12</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="Q34" t="n">
-        <v>66</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>34</v>
+        <v>15305</v>
       </c>
       <c r="B35" t="n">
         <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D35" t="n">
-        <v>-12</v>
+        <v>-6</v>
       </c>
       <c r="E35" t="n">
         <v>8</v>
@@ -2317,10 +2327,10 @@
         <v>8</v>
       </c>
       <c r="H35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J35" t="n">
         <v>8</v>
@@ -2332,92 +2342,92 @@
         <v>8</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N35" t="n">
-        <v>-12</v>
+        <v>4</v>
       </c>
       <c r="O35" t="n">
         <v>8</v>
       </c>
       <c r="P35" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q35" t="n">
-        <v>56</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>35</v>
+        <v>15308</v>
       </c>
       <c r="B36" t="n">
-        <v>-6</v>
+        <v>4</v>
       </c>
       <c r="C36" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>-12</v>
       </c>
       <c r="E36" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
         <v>4</v>
       </c>
       <c r="G36" t="n">
+        <v>8</v>
+      </c>
+      <c r="H36" t="n">
+        <v>7</v>
+      </c>
+      <c r="I36" t="n">
+        <v>4</v>
+      </c>
+      <c r="J36" t="n">
         <v>-2</v>
       </c>
-      <c r="H36" t="n">
-        <v>6</v>
-      </c>
-      <c r="I36" t="n">
-        <v>-1</v>
-      </c>
-      <c r="J36" t="n">
-        <v>6</v>
-      </c>
       <c r="K36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L36" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M36" t="n">
-        <v>3</v>
+        <v>-12</v>
       </c>
       <c r="N36" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P36" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q36" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>36</v>
+        <v>15309</v>
       </c>
       <c r="B37" t="n">
         <v>8</v>
       </c>
       <c r="C37" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E37" t="n">
         <v>8</v>
       </c>
       <c r="F37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G37" t="n">
         <v>8</v>
@@ -2426,45 +2436,45 @@
         <v>5</v>
       </c>
       <c r="I37" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K37" t="n">
         <v>8</v>
       </c>
       <c r="L37" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M37" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N37" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="O37" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="P37" t="n">
         <v>6</v>
       </c>
       <c r="Q37" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>37</v>
+        <v>15310</v>
       </c>
       <c r="B38" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D38" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E38" t="n">
         <v>8</v>
@@ -2473,50 +2483,48 @@
         <v>7</v>
       </c>
       <c r="G38" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H38" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I38" t="n">
-        <v>4</v>
+        <v>-8</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K38" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L38" t="n">
-        <v>6</v>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>8</v>
+      </c>
+      <c r="M38" t="n">
+        <v>8</v>
       </c>
       <c r="N38" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P38" t="n">
         <v>5</v>
       </c>
       <c r="Q38" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>38</v>
+        <v>15311</v>
       </c>
       <c r="B39" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C39" t="n">
-        <v>-12</v>
+        <v>4</v>
       </c>
       <c r="D39" t="n">
         <v>8</v>
@@ -2525,16 +2533,16 @@
         <v>8</v>
       </c>
       <c r="F39" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G39" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="H39" t="n">
         <v>8</v>
       </c>
       <c r="I39" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J39" t="n">
         <v>8</v>
@@ -2546,7 +2554,7 @@
         <v>8</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N39" t="n">
         <v>8</v>
@@ -2554,25 +2562,27 @@
       <c r="O39" t="n">
         <v>8</v>
       </c>
-      <c r="P39" t="n">
-        <v>6</v>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="Q39" t="n">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>39</v>
+        <v>15312</v>
       </c>
       <c r="B40" t="n">
         <v>8</v>
       </c>
       <c r="C40" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E40" t="n">
         <v>8</v>
@@ -2581,48 +2591,48 @@
         <v>8</v>
       </c>
       <c r="G40" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H40" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J40" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K40" t="n">
         <v>8</v>
       </c>
       <c r="L40" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M40" t="n">
-        <v>6</v>
+        <v>-12</v>
       </c>
       <c r="N40" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O40" t="n">
         <v>8</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q40" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>40</v>
+        <v>15313</v>
       </c>
       <c r="B41" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D41" t="n">
         <v>6</v>
@@ -2631,72 +2641,74 @@
         <v>8</v>
       </c>
       <c r="F41" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G41" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="H41" t="n">
-        <v>-6</v>
+        <v>8</v>
       </c>
       <c r="I41" t="n">
-        <v>-7</v>
+        <v>4</v>
       </c>
       <c r="J41" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="L41" t="n">
-        <v>5</v>
-      </c>
-      <c r="M41" t="n">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="N41" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O41" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P41" t="n">
-        <v>-12</v>
+        <v>5</v>
       </c>
       <c r="Q41" t="n">
-        <v>20</v>
+        <v>87</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>41</v>
+        <v>15314</v>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D42" t="n">
         <v>6</v>
       </c>
       <c r="E42" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F42" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G42" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H42" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I42" t="n">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="J42" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K42" t="n">
         <v>8</v>
@@ -2705,54 +2717,54 @@
         <v>4</v>
       </c>
       <c r="M42" t="n">
-        <v>4</v>
+        <v>-12</v>
       </c>
       <c r="N42" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O42" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P42" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q42" t="n">
-        <v>82</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>42</v>
+        <v>15315</v>
       </c>
       <c r="B43" t="n">
         <v>8</v>
       </c>
       <c r="C43" t="n">
-        <v>6</v>
+        <v>-12</v>
       </c>
       <c r="D43" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="E43" t="n">
         <v>8</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="G43" t="n">
         <v>8</v>
       </c>
       <c r="H43" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I43" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J43" t="n">
-        <v>-2</v>
+        <v>8</v>
       </c>
       <c r="K43" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L43" t="n">
         <v>8</v>
@@ -2764,24 +2776,24 @@
         <v>8</v>
       </c>
       <c r="O43" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q43" t="n">
-        <v>82</v>
+        <v>47</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>43</v>
+        <v>15316</v>
       </c>
       <c r="B44" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>-6</v>
       </c>
       <c r="D44" t="n">
         <v>5</v>
@@ -2790,160 +2802,162 @@
         <v>8</v>
       </c>
       <c r="F44" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G44" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H44" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I44" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J44" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K44" t="n">
         <v>8</v>
       </c>
       <c r="L44" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M44" t="n">
-        <v>7</v>
+        <v>-2</v>
       </c>
       <c r="N44" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O44" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Q44" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>44</v>
+        <v>15317</v>
       </c>
       <c r="B45" t="n">
-        <v>8</v>
+        <v>-2</v>
       </c>
       <c r="C45" t="n">
-        <v>-12</v>
+        <v>6</v>
       </c>
       <c r="D45" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="E45" t="n">
         <v>8</v>
       </c>
       <c r="F45" t="n">
-        <v>-6</v>
+        <v>7</v>
       </c>
       <c r="G45" t="n">
         <v>8</v>
       </c>
       <c r="H45" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I45" t="n">
-        <v>8</v>
-      </c>
-      <c r="J45" t="n">
-        <v>8</v>
+        <v>6</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="K45" t="n">
         <v>8</v>
       </c>
       <c r="L45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M45" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N45" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O45" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P45" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q45" t="n">
-        <v>79</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>45</v>
+        <v>15318</v>
       </c>
       <c r="B46" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C46" t="n">
         <v>8</v>
       </c>
       <c r="D46" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E46" t="n">
         <v>8</v>
       </c>
       <c r="F46" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G46" t="n">
-        <v>7</v>
+        <v>-12</v>
       </c>
       <c r="H46" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I46" t="n">
-        <v>-4</v>
+        <v>4</v>
       </c>
       <c r="J46" t="n">
         <v>8</v>
       </c>
       <c r="K46" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L46" t="n">
         <v>8</v>
       </c>
       <c r="M46" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="N46" t="n">
         <v>4</v>
       </c>
       <c r="O46" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q46" t="n">
-        <v>93</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>46</v>
+        <v>15320</v>
       </c>
       <c r="B47" t="n">
         <v>8</v>
       </c>
       <c r="C47" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="D47" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E47" t="n">
         <v>8</v>
@@ -2955,257 +2969,257 @@
         <v>8</v>
       </c>
       <c r="H47" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J47" t="n">
         <v>8</v>
       </c>
       <c r="K47" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L47" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M47" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N47" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O47" t="n">
         <v>8</v>
       </c>
       <c r="P47" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q47" t="n">
-        <v>87</v>
+        <v>103</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
+        <v>15321</v>
+      </c>
+      <c r="B48" t="n">
+        <v>8</v>
+      </c>
+      <c r="C48" t="n">
+        <v>6</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-6</v>
+      </c>
+      <c r="E48" t="n">
+        <v>8</v>
+      </c>
+      <c r="F48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="G48" t="n">
+        <v>8</v>
+      </c>
+      <c r="H48" t="n">
+        <v>4</v>
+      </c>
+      <c r="I48" t="n">
+        <v>7</v>
+      </c>
+      <c r="J48" t="n">
+        <v>4</v>
+      </c>
+      <c r="K48" t="n">
+        <v>8</v>
+      </c>
+      <c r="L48" t="n">
+        <v>4</v>
+      </c>
+      <c r="M48" t="n">
+        <v>-6</v>
+      </c>
+      <c r="N48" t="n">
+        <v>6</v>
+      </c>
+      <c r="O48" t="n">
+        <v>6</v>
+      </c>
+      <c r="P48" t="n">
+        <v>-7</v>
+      </c>
+      <c r="Q48" t="n">
         <v>47</v>
-      </c>
-      <c r="B48" t="n">
-        <v>8</v>
-      </c>
-      <c r="C48" t="n">
-        <v>4</v>
-      </c>
-      <c r="D48" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" t="n">
-        <v>8</v>
-      </c>
-      <c r="F48" t="n">
-        <v>6</v>
-      </c>
-      <c r="G48" t="n">
-        <v>8</v>
-      </c>
-      <c r="H48" t="n">
-        <v>5</v>
-      </c>
-      <c r="I48" t="n">
-        <v>7</v>
-      </c>
-      <c r="J48" t="n">
-        <v>5</v>
-      </c>
-      <c r="K48" t="n">
-        <v>8</v>
-      </c>
-      <c r="L48" t="n">
-        <v>8</v>
-      </c>
-      <c r="M48" t="n">
-        <v>8</v>
-      </c>
-      <c r="N48" t="n">
-        <v>6</v>
-      </c>
-      <c r="O48" t="n">
-        <v>7</v>
-      </c>
-      <c r="P48" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>90</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>48</v>
+        <v>15322</v>
       </c>
       <c r="B49" t="n">
         <v>8</v>
       </c>
       <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-12</v>
+      </c>
+      <c r="E49" t="n">
+        <v>8</v>
+      </c>
+      <c r="F49" t="n">
+        <v>6</v>
+      </c>
+      <c r="G49" t="n">
+        <v>8</v>
+      </c>
+      <c r="H49" t="n">
+        <v>6</v>
+      </c>
+      <c r="I49" t="n">
+        <v>4</v>
+      </c>
+      <c r="J49" t="n">
+        <v>8</v>
+      </c>
+      <c r="K49" t="n">
+        <v>8</v>
+      </c>
+      <c r="L49" t="n">
+        <v>8</v>
+      </c>
+      <c r="M49" t="n">
         <v>-6</v>
       </c>
-      <c r="D49" t="n">
-        <v>5</v>
-      </c>
-      <c r="E49" t="n">
-        <v>8</v>
-      </c>
-      <c r="F49" t="n">
-        <v>8</v>
-      </c>
-      <c r="G49" t="n">
-        <v>8</v>
-      </c>
-      <c r="H49" t="n">
-        <v>7</v>
-      </c>
-      <c r="I49" t="n">
-        <v>5</v>
-      </c>
-      <c r="J49" t="n">
-        <v>7</v>
-      </c>
-      <c r="K49" t="n">
-        <v>8</v>
-      </c>
-      <c r="L49" t="n">
-        <v>8</v>
-      </c>
-      <c r="M49" t="n">
-        <v>-2</v>
-      </c>
       <c r="N49" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O49" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P49" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q49" t="n">
-        <v>83</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>49</v>
+        <v>15324</v>
       </c>
       <c r="B50" t="n">
-        <v>8</v>
+        <v>-7</v>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D50" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="E50" t="n">
         <v>8</v>
       </c>
       <c r="F50" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G50" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H50" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I50" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J50" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K50" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L50" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M50" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N50" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O50" t="n">
         <v>8</v>
       </c>
       <c r="P50" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="Q50" t="n">
-        <v>110</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>50</v>
+        <v>15325</v>
       </c>
       <c r="B51" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C51" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D51" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E51" t="n">
         <v>8</v>
       </c>
       <c r="F51" t="n">
-        <v>-8</v>
+        <v>3</v>
       </c>
       <c r="G51" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H51" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I51" t="n">
+        <v>5</v>
+      </c>
+      <c r="J51" t="n">
+        <v>4</v>
+      </c>
+      <c r="K51" t="n">
+        <v>8</v>
+      </c>
+      <c r="L51" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M51" t="n">
         <v>3</v>
       </c>
-      <c r="J51" t="n">
-        <v>2</v>
-      </c>
-      <c r="K51" t="n">
-        <v>8</v>
-      </c>
-      <c r="L51" t="n">
-        <v>8</v>
-      </c>
-      <c r="M51" t="n">
-        <v>6</v>
-      </c>
       <c r="N51" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O51" t="n">
         <v>4</v>
       </c>
       <c r="P51" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q51" t="n">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>51</v>
+        <v>15326</v>
       </c>
       <c r="B52" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C52" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D52" t="n">
         <v>-12</v>
@@ -3220,65 +3234,63 @@
         <v>8</v>
       </c>
       <c r="H52" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I52" t="n">
         <v>4</v>
       </c>
       <c r="J52" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="K52" t="n">
         <v>8</v>
       </c>
       <c r="L52" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M52" t="n">
-        <v>6</v>
+        <v>-12</v>
       </c>
       <c r="N52" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="O52" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P52" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="Q52" t="n">
-        <v>56</v>
+        <v>32</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>52</v>
+        <v>15327</v>
       </c>
       <c r="B53" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C53" t="n">
-        <v>8</v>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="D53" t="n">
+        <v>8</v>
       </c>
       <c r="E53" t="n">
         <v>8</v>
       </c>
       <c r="F53" t="n">
-        <v>-2</v>
+        <v>-6</v>
       </c>
       <c r="G53" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H53" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I53" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J53" t="n">
         <v>8</v>
@@ -3287,29 +3299,27 @@
         <v>8</v>
       </c>
       <c r="L53" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M53" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>8</v>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="O53" t="n">
+        <v>7</v>
       </c>
       <c r="P53" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q53" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>53</v>
+        <v>15328</v>
       </c>
       <c r="B54" t="n">
         <v>8</v>
@@ -3345,7 +3355,7 @@
         <v>8</v>
       </c>
       <c r="M54" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="N54" t="n">
         <v>8</v>
@@ -3357,12 +3367,12 @@
         <v>5</v>
       </c>
       <c r="Q54" t="n">
-        <v>64</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>54</v>
+        <v>15330</v>
       </c>
       <c r="B55" t="n">
         <v>8</v>
@@ -3370,26 +3380,28 @@
       <c r="C55" t="n">
         <v>8</v>
       </c>
-      <c r="D55" t="n">
-        <v>4</v>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="E55" t="n">
         <v>8</v>
       </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="G55" t="n">
         <v>8</v>
       </c>
       <c r="H55" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I55" t="n">
         <v>8</v>
       </c>
       <c r="J55" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K55" t="n">
         <v>8</v>
@@ -3398,83 +3410,85 @@
         <v>8</v>
       </c>
       <c r="M55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N55" t="n">
-        <v>6</v>
-      </c>
-      <c r="O55" t="n">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="P55" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q55" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>55</v>
+        <v>15331</v>
       </c>
       <c r="B56" t="n">
-        <v>7</v>
+        <v>-6</v>
       </c>
       <c r="C56" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D56" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E56" t="n">
         <v>8</v>
       </c>
       <c r="F56" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>8</v>
+        <v>-2</v>
       </c>
       <c r="H56" t="n">
         <v>6</v>
       </c>
       <c r="I56" t="n">
-        <v>8</v>
+        <v>-1</v>
       </c>
       <c r="J56" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K56" t="n">
         <v>8</v>
       </c>
       <c r="L56" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M56" t="n">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="N56" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O56" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P56" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q56" t="n">
-        <v>98</v>
+        <v>40</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>56</v>
+        <v>15333</v>
       </c>
       <c r="B57" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C57" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D57" t="n">
         <v>8</v>
@@ -3483,245 +3497,219 @@
         <v>8</v>
       </c>
       <c r="F57" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G57" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H57" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I57" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J57" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K57" t="n">
         <v>8</v>
       </c>
       <c r="L57" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M57" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="N57" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O57" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="P57" t="n">
         <v>4</v>
       </c>
       <c r="Q57" t="n">
-        <v>71</v>
+        <v>116</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>57</v>
+        <v>15334</v>
       </c>
       <c r="B58" t="n">
+        <v>8</v>
+      </c>
+      <c r="C58" t="n">
+        <v>8</v>
+      </c>
+      <c r="D58" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E58" t="n">
+        <v>8</v>
+      </c>
+      <c r="F58" t="n">
+        <v>8</v>
+      </c>
+      <c r="G58" t="n">
+        <v>5</v>
+      </c>
+      <c r="H58" t="n">
+        <v>6</v>
+      </c>
+      <c r="I58" t="n">
         <v>0</v>
       </c>
-      <c r="C58" t="n">
-        <v>8</v>
-      </c>
-      <c r="D58" t="n">
-        <v>4</v>
-      </c>
-      <c r="E58" t="n">
-        <v>8</v>
-      </c>
-      <c r="F58" t="n">
-        <v>8</v>
-      </c>
-      <c r="G58" t="n">
-        <v>8</v>
-      </c>
-      <c r="H58" t="n">
-        <v>4</v>
-      </c>
-      <c r="I58" t="n">
-        <v>3</v>
-      </c>
       <c r="J58" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K58" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L58" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M58" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N58" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O58" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P58" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Q58" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>15336</v>
+      </c>
+      <c r="B59" t="n">
+        <v>8</v>
+      </c>
+      <c r="C59" t="n">
+        <v>8</v>
+      </c>
+      <c r="D59" t="n">
+        <v>8</v>
       </c>
       <c r="E59" t="n">
-        <v>4</v>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>8</v>
+      </c>
+      <c r="F59" t="n">
+        <v>6</v>
+      </c>
+      <c r="G59" t="n">
+        <v>8</v>
+      </c>
+      <c r="H59" t="n">
+        <v>6</v>
+      </c>
+      <c r="I59" t="n">
+        <v>8</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" t="n">
+        <v>8</v>
+      </c>
+      <c r="L59" t="n">
+        <v>8</v>
       </c>
       <c r="M59" t="n">
-        <v>-12</v>
-      </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="O59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="P59" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>6</v>
+      </c>
+      <c r="N59" t="n">
+        <v>8</v>
+      </c>
+      <c r="O59" t="n">
+        <v>8</v>
+      </c>
+      <c r="P59" t="n">
+        <v>5</v>
       </c>
       <c r="Q59" t="n">
-        <v>-8</v>
+        <v>103</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>59</v>
+        <v>15337</v>
       </c>
       <c r="B60" t="n">
-        <v>-7</v>
+        <v>8</v>
       </c>
       <c r="C60" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D60" t="n">
-        <v>-12</v>
+        <v>4</v>
       </c>
       <c r="E60" t="n">
         <v>8</v>
       </c>
       <c r="F60" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G60" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H60" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I60" t="n">
         <v>4</v>
       </c>
       <c r="J60" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K60" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L60" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M60" t="n">
-        <v>4</v>
+        <v>-12</v>
       </c>
       <c r="N60" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O60" t="n">
         <v>8</v>
       </c>
       <c r="P60" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="Q60" t="n">
-        <v>45</v>
+        <v>84</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>60</v>
+        <v>15338</v>
       </c>
       <c r="B61" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C61" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D61" t="n">
-        <v>-12</v>
+        <v>8</v>
       </c>
       <c r="E61" t="n">
         <v>8</v>
       </c>
       <c r="F61" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G61" t="n">
         <v>8</v>
@@ -3730,39 +3718,39 @@
         <v>5</v>
       </c>
       <c r="I61" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J61" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K61" t="n">
         <v>8</v>
       </c>
       <c r="L61" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="M61" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N61" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O61" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P61" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q61" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>61</v>
+        <v>15342</v>
       </c>
       <c r="B62" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C62" t="n">
         <v>8</v>
@@ -3773,222 +3761,234 @@
       <c r="E62" t="n">
         <v>8</v>
       </c>
-      <c r="F62" t="n">
-        <v>8</v>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="G62" t="n">
         <v>8</v>
       </c>
       <c r="H62" t="n">
-        <v>4</v>
-      </c>
-      <c r="I62" t="n">
-        <v>4</v>
-      </c>
-      <c r="J62" t="n">
-        <v>8</v>
-      </c>
-      <c r="K62" t="n">
-        <v>8</v>
-      </c>
-      <c r="L62" t="n">
-        <v>8</v>
+        <v>8</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="M62" t="n">
-        <v>-12</v>
-      </c>
-      <c r="N62" t="n">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="O62" t="n">
         <v>8</v>
       </c>
-      <c r="P62" t="n">
-        <v>8</v>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="Q62" t="n">
-        <v>84</v>
+        <v>56</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+        <v>15343</v>
+      </c>
+      <c r="B63" t="n">
+        <v>8</v>
+      </c>
+      <c r="C63" t="n">
+        <v>-12</v>
+      </c>
+      <c r="D63" t="n">
+        <v>8</v>
       </c>
       <c r="E63" t="n">
         <v>8</v>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="O63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
-      </c>
-      <c r="P63" t="inlineStr">
-        <is>
-          <t>invalid_answer</t>
-        </is>
+      <c r="F63" t="n">
+        <v>-6</v>
+      </c>
+      <c r="G63" t="n">
+        <v>8</v>
+      </c>
+      <c r="H63" t="n">
+        <v>8</v>
+      </c>
+      <c r="I63" t="n">
+        <v>8</v>
+      </c>
+      <c r="J63" t="n">
+        <v>8</v>
+      </c>
+      <c r="K63" t="n">
+        <v>8</v>
+      </c>
+      <c r="L63" t="n">
+        <v>8</v>
+      </c>
+      <c r="M63" t="n">
+        <v>-7</v>
+      </c>
+      <c r="N63" t="n">
+        <v>8</v>
+      </c>
+      <c r="O63" t="n">
+        <v>8</v>
+      </c>
+      <c r="P63" t="n">
+        <v>8</v>
       </c>
       <c r="Q63" t="n">
-        <v>8</v>
+        <v>71</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>63</v>
+        <v>15344</v>
       </c>
       <c r="B64" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C64" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E64" t="n">
         <v>8</v>
       </c>
       <c r="F64" t="n">
+        <v>8</v>
+      </c>
+      <c r="G64" t="n">
+        <v>-12</v>
+      </c>
+      <c r="H64" t="n">
         <v>-6</v>
       </c>
-      <c r="G64" t="n">
-        <v>6</v>
-      </c>
-      <c r="H64" t="n">
-        <v>7</v>
-      </c>
       <c r="I64" t="n">
-        <v>7</v>
+        <v>-7</v>
       </c>
       <c r="J64" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K64" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="L64" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M64" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N64" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O64" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P64" t="n">
-        <v>7</v>
+        <v>-12</v>
       </c>
       <c r="Q64" t="n">
-        <v>82</v>
+        <v>20</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" t="n">
-        <v>4</v>
-      </c>
-      <c r="C65" t="n">
-        <v>4</v>
-      </c>
-      <c r="D65" t="n">
-        <v>8</v>
+        <v>15348</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="E65" t="n">
         <v>8</v>
       </c>
-      <c r="F65" t="n">
-        <v>4</v>
-      </c>
-      <c r="G65" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" t="n">
-        <v>8</v>
-      </c>
-      <c r="I65" t="n">
-        <v>8</v>
-      </c>
-      <c r="J65" t="n">
-        <v>8</v>
-      </c>
-      <c r="K65" t="n">
-        <v>8</v>
-      </c>
-      <c r="L65" t="n">
-        <v>8</v>
-      </c>
-      <c r="M65" t="n">
-        <v>4</v>
-      </c>
-      <c r="N65" t="n">
-        <v>8</v>
-      </c>
-      <c r="O65" t="n">
-        <v>8</v>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>invalid_answer</t>
+        </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
@@ -3996,15 +3996,15 @@
         </is>
       </c>
       <c r="Q65" t="n">
-        <v>88</v>
+        <v>8</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>65</v>
+        <v>15349</v>
       </c>
       <c r="B66" t="n">
-        <v>-6</v>
+        <v>8</v>
       </c>
       <c r="C66" t="n">
         <v>4</v>
@@ -4016,28 +4016,28 @@
         <v>8</v>
       </c>
       <c r="F66" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G66" t="n">
         <v>8</v>
       </c>
       <c r="H66" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I66" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J66" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K66" t="n">
         <v>8</v>
       </c>
       <c r="L66" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M66" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="N66" t="n">
         <v>8</v>
@@ -4046,39 +4046,39 @@
         <v>8</v>
       </c>
       <c r="P66" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q66" t="n">
-        <v>84</v>
+        <v>111</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>66</v>
+        <v>15351</v>
       </c>
       <c r="B67" t="n">
         <v>8</v>
       </c>
       <c r="C67" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D67" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E67" t="n">
         <v>8</v>
       </c>
       <c r="F67" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G67" t="n">
         <v>8</v>
       </c>
       <c r="H67" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I67" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J67" t="n">
         <v>8</v>
@@ -4090,10 +4090,10 @@
         <v>8</v>
       </c>
       <c r="M67" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N67" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="O67" t="n">
         <v>8</v>
@@ -4102,27 +4102,27 @@
         <v>8</v>
       </c>
       <c r="Q67" t="n">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>67</v>
+        <v>15352</v>
       </c>
       <c r="B68" t="n">
         <v>8</v>
       </c>
       <c r="C68" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D68" t="n">
-        <v>8</v>
+        <v>-12</v>
       </c>
       <c r="E68" t="n">
         <v>8</v>
       </c>
       <c r="F68" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G68" t="n">
         <v>8</v>
@@ -4131,10 +4131,10 @@
         <v>4</v>
       </c>
       <c r="I68" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J68" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K68" t="n">
         <v>8</v>
@@ -4143,7 +4143,7 @@
         <v>8</v>
       </c>
       <c r="M68" t="n">
-        <v>4</v>
+        <v>-12</v>
       </c>
       <c r="N68" t="n">
         <v>8</v>
@@ -4152,21 +4152,21 @@
         <v>8</v>
       </c>
       <c r="P68" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q68" t="n">
-        <v>106</v>
+        <v>60</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>68</v>
+        <v>15353</v>
       </c>
       <c r="B69" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C69" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D69" t="n">
         <v>8</v>
@@ -4181,22 +4181,22 @@
         <v>8</v>
       </c>
       <c r="H69" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I69" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J69" t="n">
-        <v>8</v>
+        <v>-2</v>
       </c>
       <c r="K69" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L69" t="n">
         <v>8</v>
       </c>
       <c r="M69" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N69" t="n">
         <v>8</v>
@@ -4205,10 +4205,10 @@
         <v>8</v>
       </c>
       <c r="P69" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Q69" t="n">
-        <v>108</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>